<commit_message>
doc: update how to use section to reflectr new approach
</commit_message>
<xml_diff>
--- a/data/PPA_scenario_definition.xlsx
+++ b/data/PPA_scenario_definition.xlsx
@@ -1529,7 +1529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C70"/>
+  <dimension ref="B1:C70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1874,44 +1874,40 @@
     <row r="59" ht="16" customHeight="1">
       <c r="B59" s="31" t="inlineStr">
         <is>
-          <t>1. Upload this file to your Google Drive.</t>
+          <t>1. In Google Colab, open the file browser (folder icon in the left sidebar).</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="B60" s="31" t="inlineStr">
         <is>
-          <t>2. Note the path within your Drive (root = just the filename; subfolder = e.g. "pypsa-ppa/PPA_scenario_definition.xlsx").</t>
+          <t>2. Navigate into the data/ folder (or create it if it doesn't exist).</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="B61" s="31" t="inlineStr">
         <is>
-          <t>3. In the notebook's scenario loading cell, set _GDRIVE_XLSX_PATH to that path.</t>
+          <t>3. Right-click inside data/ and choose Upload, then select PPA_scenario_definition.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="B62" s="32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   _GDRIVE_XLSX_PATH = "PPA_scenario_definition.xlsx"</t>
+          <t>4. The notebook will find the file automatically at data/PPA_scenario_definition.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="B63" s="31" t="inlineStr">
         <is>
-          <t>4. Run the cell — it calls drive.mount() to connect your Drive, then reads the file directly.</t>
+          <t>5. Re-run the notebook from the scenario loading cell to pick up any edits.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
-      <c r="B64" s="31" t="inlineStr">
-        <is>
-          <t>5. Re-run the notebook from the scenario loading cell to pick up any edits to the Excel.</t>
-        </is>
-      </c>
+      <c r="B64" s="31" t="inlineStr"/>
     </row>
     <row r="65" ht="7" customHeight="1"/>
     <row r="66" ht="16" customHeight="1">

</xml_diff>